<commit_message>
stundenlang fehler gesucht und debugged
</commit_message>
<xml_diff>
--- a/Input_data/Muster_Honorarrechnung-Lehrkräfte_pytest.xlsx
+++ b/Input_data/Muster_Honorarrechnung-Lehrkräfte_pytest.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\domin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projekt_kalender_pro_beruf\Input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504D93D1-BB43-4212-BA9F-3ADF663CD0BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A1C2AC-D7A0-4AAE-9CB0-5824623EAAC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Rechnungsvorlage Honorar" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Rechnungsvorlage Honorar'!$A$1:$E$65</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Rechnungsvorlage Honorar'!$A$1:$E$74</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -167,9 +167,6 @@
     <t>01/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">für die unten aufgeführten Leistungen als Honorardozent:in im Projekt Assistierte Ausbildung AsA VIII berechne ich Ihnen wie folgt: </t>
-  </si>
-  <si>
     <t>04.02.2026 bis 26.02.2026</t>
   </si>
   <si>
@@ -192,6 +189,9 @@
   </si>
   <si>
     <t>SumUp Limited</t>
+  </si>
+  <si>
+    <t xml:space="preserve">für die unten aufgeführten Leistungen für den Stütz- und Förderunterricht in der Ausbildungsassistenz im Projekt Assistierte Ausbildung AsA VIII berechne ich Ihnen wie folgt: </t>
   </si>
 </sst>
 </file>
@@ -839,7 +839,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.3828125" defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.07421875" style="1" customWidth="1"/>
@@ -865,7 +865,7 @@
         <v>17</v>
       </c>
       <c r="B2" s="46" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="10"/>
@@ -876,7 +876,7 @@
         <v>14</v>
       </c>
       <c r="B3" s="46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="10"/>
@@ -888,7 +888,7 @@
         <v>15</v>
       </c>
       <c r="B4" s="46" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="10"/>
@@ -899,7 +899,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="48" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="10"/>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B6" s="46" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="10"/>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B24" s="18"/>
       <c r="C24" s="27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
@@ -1066,7 +1066,7 @@
     </row>
     <row r="29" spans="1:9" ht="34.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="52" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B29" s="52"/>
       <c r="C29" s="52"/>
@@ -1111,7 +1111,7 @@
       <c r="C33" s="26"/>
       <c r="D33" s="16"/>
       <c r="E33" s="37">
-        <f t="shared" ref="E33:E48" si="0">ROUND(B33*$D$32,2)</f>
+        <f t="shared" ref="E33:E57" si="0">ROUND(B33*$D$32,2)</f>
         <v>0</v>
       </c>
     </row>
@@ -1265,162 +1265,252 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" s="7" customFormat="1" ht="14.6" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A49" s="50" t="s">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A49" s="44"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A50" s="44"/>
+      <c r="B50" s="21"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A51" s="44"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52" s="44"/>
+      <c r="B52" s="21"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A53" s="44"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54" s="44"/>
+      <c r="B54" s="21"/>
+      <c r="C54" s="22"/>
+      <c r="D54" s="23"/>
+      <c r="E54" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A55" s="44"/>
+      <c r="B55" s="21"/>
+      <c r="C55" s="22"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" s="44"/>
+      <c r="B56" s="21"/>
+      <c r="C56" s="22"/>
+      <c r="D56" s="23"/>
+      <c r="E56" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A57" s="44"/>
+      <c r="B57" s="21"/>
+      <c r="C57" s="22"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="37">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" s="7" customFormat="1" ht="14.6" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A58" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="B49" s="51"/>
-      <c r="C49" s="51"/>
-      <c r="D49" s="24"/>
-      <c r="E49" s="38">
-        <f>SUM(E32:E48)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B50" s="3"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="8"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="9"/>
-      <c r="I50" s="9"/>
-    </row>
-    <row r="51" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
+      <c r="B58" s="51"/>
+      <c r="C58" s="51"/>
+      <c r="D58" s="24"/>
+      <c r="E58" s="38">
+        <f>SUM(E32:E57)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B59" s="3"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="13"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="9"/>
+      <c r="I59" s="9"/>
+    </row>
+    <row r="60" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B51" s="2"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-    </row>
-    <row r="52" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A53" s="1" t="s">
+      <c r="B60" s="2"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
+    </row>
+    <row r="61" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="14"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A62" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B53" s="20"/>
-      <c r="C53" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
+      <c r="B62" s="20"/>
+      <c r="C62" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A63" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="40" t="s">
-        <v>33</v>
-      </c>
-      <c r="D54" s="12"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A55" s="1" t="s">
+      <c r="B63" s="20"/>
+      <c r="C63" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="D63" s="12"/>
+      <c r="E63" s="10"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A64" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B55" s="3"/>
-      <c r="C55" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="D55" s="12"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="3"/>
-      <c r="I55" s="3"/>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B56" s="3"/>
-      <c r="C56" s="6"/>
-      <c r="D56" s="54"/>
-      <c r="E56" s="54"/>
-      <c r="F56" s="6"/>
-      <c r="G56" s="6"/>
-      <c r="H56" s="3"/>
-      <c r="I56" s="3"/>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="D57" s="53" t="s">
+      <c r="B64" s="3"/>
+      <c r="C64" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D64" s="12"/>
+      <c r="E64" s="10"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B65" s="3"/>
+      <c r="C65" s="6"/>
+      <c r="D65" s="54"/>
+      <c r="E65" s="54"/>
+      <c r="F65" s="6"/>
+      <c r="G65" s="6"/>
+      <c r="H65" s="3"/>
+      <c r="I65" s="3"/>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D66" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="E57" s="53"/>
-      <c r="F57" s="6"/>
-      <c r="G57" s="6"/>
-      <c r="H57" s="3"/>
-      <c r="I57" s="3"/>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="D58" s="33"/>
-      <c r="E58" s="33"/>
-      <c r="F58" s="6"/>
-      <c r="G58" s="6"/>
-      <c r="H58" s="3"/>
-      <c r="I58" s="3"/>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="D59" s="33"/>
-      <c r="E59" s="33"/>
-      <c r="F59" s="6"/>
-      <c r="G59" s="6"/>
-      <c r="H59" s="3"/>
-      <c r="I59" s="3"/>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="D60" s="33"/>
-      <c r="E60" s="33"/>
-      <c r="F60" s="6"/>
-      <c r="G60" s="6"/>
-      <c r="H60" s="3"/>
-      <c r="I60" s="3"/>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B61" s="3"/>
-      <c r="C61" s="6"/>
-      <c r="D61" s="1"/>
-      <c r="E61" s="12"/>
-      <c r="F61" s="6"/>
-      <c r="G61" s="6"/>
-      <c r="H61" s="3"/>
-      <c r="I61" s="3"/>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A62" s="32"/>
-      <c r="B62" s="32"/>
-      <c r="C62" s="11"/>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A63" s="34" t="s">
+      <c r="E66" s="53"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="6"/>
+      <c r="H66" s="3"/>
+      <c r="I66" s="3"/>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D67" s="33"/>
+      <c r="E67" s="33"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6"/>
+      <c r="H67" s="3"/>
+      <c r="I67" s="3"/>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D68" s="33"/>
+      <c r="E68" s="33"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="6"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D69" s="33"/>
+      <c r="E69" s="33"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B70" s="3"/>
+      <c r="C70" s="6"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="12"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A71" s="32"/>
+      <c r="B71" s="32"/>
+      <c r="C71" s="11"/>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A72" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="B63" s="34"/>
-      <c r="C63" s="34"/>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A64" s="42" t="s">
+      <c r="B72" s="34"/>
+      <c r="C72" s="34"/>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A73" s="42" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1428,10 +1518,10 @@
   <mergeCells count="7">
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:I10"/>
-    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A58:C58"/>
     <mergeCell ref="A29:E29"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D65:E65"/>
     <mergeCell ref="G24:I24"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>